<commit_message>
Add 1K (1024 tok) and 2K (2048 tok) k6 online <50ms saturation sweeps alongside 1KB/2KB payloads
</commit_message>
<xml_diff>
--- a/models/JinaEmbedding/vLLM/megakernel/ATP_AIC2_Benchmarks_TPU_v6e_FP32_Megakernel_vs_L4_and_Baselines.xlsx
+++ b/models/JinaEmbedding/vLLM/megakernel/ATP_AIC2_Benchmarks_TPU_v6e_FP32_Megakernel_vs_L4_and_Baselines.xlsx
@@ -2,10 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="k6_RPS_Sub50ms_1KB_2KB" sheetId="1" r:id="rId1"/>
+    <sheet name="k6_Online_Sub50ms_1K_2K" sheetId="1" r:id="rId1"/>
     <sheet name="Batch_1K_2K_Tokens_Only" sheetId="2" r:id="rId2"/>
-    <sheet name="k6_Concurrency_1KB_2KB" sheetId="3" r:id="rId3"/>
-    <sheet name="MultiPrompt_Batch_1KB_2KB" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -22,7 +20,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Payload</t>
+          <t>Payload / Token Length</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -1209,6 +1207,852 @@
         </is>
       </c>
       <c r="M25" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1K_Tokens_1024</t>
+        </is>
+      </c>
+      <c r="B26" s="0">
+        <v>60</v>
+      </c>
+      <c r="C26" s="0">
+        <v>60.0</v>
+      </c>
+      <c r="D26" s="0">
+        <v>9.6</v>
+      </c>
+      <c r="E26" s="0">
+        <v>10.1</v>
+      </c>
+      <c r="F26" s="0">
+        <v>10.3</v>
+      </c>
+      <c r="G26" s="0">
+        <v>11.4</v>
+      </c>
+      <c r="H26" s="0">
+        <v>9.7</v>
+      </c>
+      <c r="I26" s="0">
+        <v>9.0</v>
+      </c>
+      <c r="J26" s="0">
+        <v>13.6</v>
+      </c>
+      <c r="K26" s="0">
+        <v>0</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1K_Tokens_1024</t>
+        </is>
+      </c>
+      <c r="B27" s="0">
+        <v>80</v>
+      </c>
+      <c r="C27" s="0">
+        <v>80.0</v>
+      </c>
+      <c r="D27" s="0">
+        <v>9.2</v>
+      </c>
+      <c r="E27" s="0">
+        <v>9.7</v>
+      </c>
+      <c r="F27" s="0">
+        <v>10.2</v>
+      </c>
+      <c r="G27" s="0">
+        <v>11.8</v>
+      </c>
+      <c r="H27" s="0">
+        <v>9.4</v>
+      </c>
+      <c r="I27" s="0">
+        <v>8.8</v>
+      </c>
+      <c r="J27" s="0">
+        <v>17.3</v>
+      </c>
+      <c r="K27" s="0">
+        <v>0</v>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1K_Tokens_1024</t>
+        </is>
+      </c>
+      <c r="B28" s="0">
+        <v>100</v>
+      </c>
+      <c r="C28" s="0">
+        <v>100.0</v>
+      </c>
+      <c r="D28" s="0">
+        <v>9.4</v>
+      </c>
+      <c r="E28" s="0">
+        <v>10.1</v>
+      </c>
+      <c r="F28" s="0">
+        <v>10.7</v>
+      </c>
+      <c r="G28" s="0">
+        <v>15.3</v>
+      </c>
+      <c r="H28" s="0">
+        <v>9.6</v>
+      </c>
+      <c r="I28" s="0">
+        <v>9.1</v>
+      </c>
+      <c r="J28" s="0">
+        <v>16.5</v>
+      </c>
+      <c r="K28" s="0">
+        <v>0</v>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1K_Tokens_1024</t>
+        </is>
+      </c>
+      <c r="B29" s="0">
+        <v>120</v>
+      </c>
+      <c r="C29" s="0">
+        <v>119.9</v>
+      </c>
+      <c r="D29" s="0">
+        <v>11.5</v>
+      </c>
+      <c r="E29" s="0">
+        <v>13.3</v>
+      </c>
+      <c r="F29" s="0">
+        <v>13.7</v>
+      </c>
+      <c r="G29" s="0">
+        <v>14.2</v>
+      </c>
+      <c r="H29" s="0">
+        <v>11.8</v>
+      </c>
+      <c r="I29" s="0">
+        <v>9.2</v>
+      </c>
+      <c r="J29" s="0">
+        <v>17.9</v>
+      </c>
+      <c r="K29" s="0">
+        <v>0</v>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>1K_Tokens_1024</t>
+        </is>
+      </c>
+      <c r="B30" s="0">
+        <v>140</v>
+      </c>
+      <c r="C30" s="0">
+        <v>139.9</v>
+      </c>
+      <c r="D30" s="0">
+        <v>12.1</v>
+      </c>
+      <c r="E30" s="0">
+        <v>12.6</v>
+      </c>
+      <c r="F30" s="0">
+        <v>12.9</v>
+      </c>
+      <c r="G30" s="0">
+        <v>13.6</v>
+      </c>
+      <c r="H30" s="0">
+        <v>12.0</v>
+      </c>
+      <c r="I30" s="0">
+        <v>9.7</v>
+      </c>
+      <c r="J30" s="0">
+        <v>17.7</v>
+      </c>
+      <c r="K30" s="0">
+        <v>0</v>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>1K_Tokens_1024</t>
+        </is>
+      </c>
+      <c r="B31" s="0">
+        <v>160</v>
+      </c>
+      <c r="C31" s="0">
+        <v>159.9</v>
+      </c>
+      <c r="D31" s="0">
+        <v>11.4</v>
+      </c>
+      <c r="E31" s="0">
+        <v>12.0</v>
+      </c>
+      <c r="F31" s="0">
+        <v>12.3</v>
+      </c>
+      <c r="G31" s="0">
+        <v>13.6</v>
+      </c>
+      <c r="H31" s="0">
+        <v>11.5</v>
+      </c>
+      <c r="I31" s="0">
+        <v>10.2</v>
+      </c>
+      <c r="J31" s="0">
+        <v>22.4</v>
+      </c>
+      <c r="K31" s="0">
+        <v>0</v>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>1K_Tokens_1024</t>
+        </is>
+      </c>
+      <c r="B32" s="0">
+        <v>180</v>
+      </c>
+      <c r="C32" s="0">
+        <v>179.9</v>
+      </c>
+      <c r="D32" s="0">
+        <v>11.2</v>
+      </c>
+      <c r="E32" s="0">
+        <v>16.0</v>
+      </c>
+      <c r="F32" s="0">
+        <v>21.8</v>
+      </c>
+      <c r="G32" s="0">
+        <v>34.7</v>
+      </c>
+      <c r="H32" s="0">
+        <v>12.6</v>
+      </c>
+      <c r="I32" s="0">
+        <v>10.2</v>
+      </c>
+      <c r="J32" s="0">
+        <v>39.5</v>
+      </c>
+      <c r="K32" s="0">
+        <v>0</v>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>1K_Tokens_1024</t>
+        </is>
+      </c>
+      <c r="B33" s="0">
+        <v>200</v>
+      </c>
+      <c r="C33" s="0">
+        <v>199.6</v>
+      </c>
+      <c r="D33" s="0">
+        <v>47.2</v>
+      </c>
+      <c r="E33" s="0">
+        <v>80.0</v>
+      </c>
+      <c r="F33" s="0">
+        <v>86.1</v>
+      </c>
+      <c r="G33" s="0">
+        <v>92.3</v>
+      </c>
+      <c r="H33" s="0">
+        <v>48.4</v>
+      </c>
+      <c r="I33" s="0">
+        <v>13.0</v>
+      </c>
+      <c r="J33" s="0">
+        <v>96.5</v>
+      </c>
+      <c r="K33" s="0">
+        <v>0</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>EXCEEDS 50ms</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2K_Tokens_2048</t>
+        </is>
+      </c>
+      <c r="B34" s="0">
+        <v>40</v>
+      </c>
+      <c r="C34" s="0">
+        <v>40.0</v>
+      </c>
+      <c r="D34" s="0">
+        <v>12.9</v>
+      </c>
+      <c r="E34" s="0">
+        <v>13.2</v>
+      </c>
+      <c r="F34" s="0">
+        <v>13.3</v>
+      </c>
+      <c r="G34" s="0">
+        <v>14.1</v>
+      </c>
+      <c r="H34" s="0">
+        <v>13.0</v>
+      </c>
+      <c r="I34" s="0">
+        <v>12.4</v>
+      </c>
+      <c r="J34" s="0">
+        <v>15.3</v>
+      </c>
+      <c r="K34" s="0">
+        <v>0</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2K_Tokens_2048</t>
+        </is>
+      </c>
+      <c r="B35" s="0">
+        <v>60</v>
+      </c>
+      <c r="C35" s="0">
+        <v>60.0</v>
+      </c>
+      <c r="D35" s="0">
+        <v>12.5</v>
+      </c>
+      <c r="E35" s="0">
+        <v>12.7</v>
+      </c>
+      <c r="F35" s="0">
+        <v>12.9</v>
+      </c>
+      <c r="G35" s="0">
+        <v>14.2</v>
+      </c>
+      <c r="H35" s="0">
+        <v>12.5</v>
+      </c>
+      <c r="I35" s="0">
+        <v>12.0</v>
+      </c>
+      <c r="J35" s="0">
+        <v>16.1</v>
+      </c>
+      <c r="K35" s="0">
+        <v>0</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2K_Tokens_2048</t>
+        </is>
+      </c>
+      <c r="B36" s="0">
+        <v>80</v>
+      </c>
+      <c r="C36" s="0">
+        <v>80.0</v>
+      </c>
+      <c r="D36" s="0">
+        <v>12.5</v>
+      </c>
+      <c r="E36" s="0">
+        <v>13.8</v>
+      </c>
+      <c r="F36" s="0">
+        <v>14.3</v>
+      </c>
+      <c r="G36" s="0">
+        <v>16.6</v>
+      </c>
+      <c r="H36" s="0">
+        <v>12.8</v>
+      </c>
+      <c r="I36" s="0">
+        <v>11.8</v>
+      </c>
+      <c r="J36" s="0">
+        <v>20.9</v>
+      </c>
+      <c r="K36" s="0">
+        <v>0</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2K_Tokens_2048</t>
+        </is>
+      </c>
+      <c r="B37" s="0">
+        <v>90</v>
+      </c>
+      <c r="C37" s="0">
+        <v>90.0</v>
+      </c>
+      <c r="D37" s="0">
+        <v>14.3</v>
+      </c>
+      <c r="E37" s="0">
+        <v>17.8</v>
+      </c>
+      <c r="F37" s="0">
+        <v>18.0</v>
+      </c>
+      <c r="G37" s="0">
+        <v>18.7</v>
+      </c>
+      <c r="H37" s="0">
+        <v>15.0</v>
+      </c>
+      <c r="I37" s="0">
+        <v>11.4</v>
+      </c>
+      <c r="J37" s="0">
+        <v>20.2</v>
+      </c>
+      <c r="K37" s="0">
+        <v>0</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2K_Tokens_2048</t>
+        </is>
+      </c>
+      <c r="B38" s="0">
+        <v>100</v>
+      </c>
+      <c r="C38" s="0">
+        <v>99.9</v>
+      </c>
+      <c r="D38" s="0">
+        <v>16.6</v>
+      </c>
+      <c r="E38" s="0">
+        <v>17.8</v>
+      </c>
+      <c r="F38" s="0">
+        <v>18.0</v>
+      </c>
+      <c r="G38" s="0">
+        <v>18.9</v>
+      </c>
+      <c r="H38" s="0">
+        <v>16.7</v>
+      </c>
+      <c r="I38" s="0">
+        <v>13.4</v>
+      </c>
+      <c r="J38" s="0">
+        <v>20.7</v>
+      </c>
+      <c r="K38" s="0">
+        <v>0</v>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2K_Tokens_2048</t>
+        </is>
+      </c>
+      <c r="B39" s="0">
+        <v>110</v>
+      </c>
+      <c r="C39" s="0">
+        <v>109.9</v>
+      </c>
+      <c r="D39" s="0">
+        <v>15.5</v>
+      </c>
+      <c r="E39" s="0">
+        <v>16.4</v>
+      </c>
+      <c r="F39" s="0">
+        <v>16.5</v>
+      </c>
+      <c r="G39" s="0">
+        <v>17.2</v>
+      </c>
+      <c r="H39" s="0">
+        <v>15.6</v>
+      </c>
+      <c r="I39" s="0">
+        <v>13.0</v>
+      </c>
+      <c r="J39" s="0">
+        <v>19.0</v>
+      </c>
+      <c r="K39" s="0">
+        <v>0</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2K_Tokens_2048</t>
+        </is>
+      </c>
+      <c r="B40" s="0">
+        <v>120</v>
+      </c>
+      <c r="C40" s="0">
+        <v>119.9</v>
+      </c>
+      <c r="D40" s="0">
+        <v>14.8</v>
+      </c>
+      <c r="E40" s="0">
+        <v>15.5</v>
+      </c>
+      <c r="F40" s="0">
+        <v>15.8</v>
+      </c>
+      <c r="G40" s="0">
+        <v>16.5</v>
+      </c>
+      <c r="H40" s="0">
+        <v>14.9</v>
+      </c>
+      <c r="I40" s="0">
+        <v>13.0</v>
+      </c>
+      <c r="J40" s="0">
+        <v>23.2</v>
+      </c>
+      <c r="K40" s="0">
+        <v>0</v>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2K_Tokens_2048</t>
+        </is>
+      </c>
+      <c r="B41" s="0">
+        <v>130</v>
+      </c>
+      <c r="C41" s="0">
+        <v>129.9</v>
+      </c>
+      <c r="D41" s="0">
+        <v>14.4</v>
+      </c>
+      <c r="E41" s="0">
+        <v>15.0</v>
+      </c>
+      <c r="F41" s="0">
+        <v>15.5</v>
+      </c>
+      <c r="G41" s="0">
+        <v>16.8</v>
+      </c>
+      <c r="H41" s="0">
+        <v>14.5</v>
+      </c>
+      <c r="I41" s="0">
+        <v>12.2</v>
+      </c>
+      <c r="J41" s="0">
+        <v>20.5</v>
+      </c>
+      <c r="K41" s="0">
+        <v>0</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2K_Tokens_2048</t>
+        </is>
+      </c>
+      <c r="B42" s="0">
+        <v>140</v>
+      </c>
+      <c r="C42" s="0">
+        <v>139.6</v>
+      </c>
+      <c r="D42" s="0">
+        <v>14.1</v>
+      </c>
+      <c r="E42" s="0">
+        <v>40.5</v>
+      </c>
+      <c r="F42" s="0">
+        <v>47.7</v>
+      </c>
+      <c r="G42" s="0">
+        <v>56.3</v>
+      </c>
+      <c r="H42" s="0">
+        <v>18.7</v>
+      </c>
+      <c r="I42" s="0">
+        <v>12.3</v>
+      </c>
+      <c r="J42" s="0">
+        <v>64.0</v>
+      </c>
+      <c r="K42" s="0">
+        <v>0</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>EXCEEDS 50ms</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>PASS (&lt;50ms)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2K_Tokens_2048</t>
+        </is>
+      </c>
+      <c r="B43" s="0">
+        <v>150</v>
+      </c>
+      <c r="C43" s="0">
+        <v>149.6</v>
+      </c>
+      <c r="D43" s="0">
+        <v>48.9</v>
+      </c>
+      <c r="E43" s="0">
+        <v>88.6</v>
+      </c>
+      <c r="F43" s="0">
+        <v>103.8</v>
+      </c>
+      <c r="G43" s="0">
+        <v>121.0</v>
+      </c>
+      <c r="H43" s="0">
+        <v>54.9</v>
+      </c>
+      <c r="I43" s="0">
+        <v>14.8</v>
+      </c>
+      <c r="J43" s="0">
+        <v>133.6</v>
+      </c>
+      <c r="K43" s="0">
+        <v>0</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>EXCEEDS 50ms</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
         <is>
           <t>PASS (&lt;50ms)</t>
         </is>
@@ -1607,578 +2451,4 @@
     </row>
   </sheetData>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="7" width="24" customWidth="1"/>
-    <col min="8" max="10" width="22" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Payload</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Concurrency (VUs)</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Achieved RPS</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>p50 (ms)</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>p90 (ms)</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>p95 (ms)</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>p99 (ms)</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>avg (ms)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1KB</t>
-        </is>
-      </c>
-      <c r="B2" s="0">
-        <v>1</v>
-      </c>
-      <c r="C2" s="0">
-        <v>101.8</v>
-      </c>
-      <c r="D2" s="0">
-        <v>9.51</v>
-      </c>
-      <c r="E2" s="0">
-        <v>10.86</v>
-      </c>
-      <c r="F2" s="0">
-        <v>11.33</v>
-      </c>
-      <c r="G2" s="0">
-        <v>12.22</v>
-      </c>
-      <c r="H2" s="0">
-        <v>9.67</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1KB</t>
-        </is>
-      </c>
-      <c r="B3" s="0">
-        <v>4</v>
-      </c>
-      <c r="C3" s="0">
-        <v>191.1</v>
-      </c>
-      <c r="D3" s="0">
-        <v>20.71</v>
-      </c>
-      <c r="E3" s="0">
-        <v>25.99</v>
-      </c>
-      <c r="F3" s="0">
-        <v>27.89</v>
-      </c>
-      <c r="G3" s="0">
-        <v>31.67</v>
-      </c>
-      <c r="H3" s="0">
-        <v>20.76</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1KB</t>
-        </is>
-      </c>
-      <c r="B4" s="0">
-        <v>8</v>
-      </c>
-      <c r="C4" s="0">
-        <v>195.36</v>
-      </c>
-      <c r="D4" s="0">
-        <v>39.31</v>
-      </c>
-      <c r="E4" s="0">
-        <v>48.42</v>
-      </c>
-      <c r="F4" s="0">
-        <v>50.1</v>
-      </c>
-      <c r="G4" s="0">
-        <v>58.71</v>
-      </c>
-      <c r="H4" s="0">
-        <v>40.77</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1KB</t>
-        </is>
-      </c>
-      <c r="B5" s="0">
-        <v>16</v>
-      </c>
-      <c r="C5" s="0">
-        <v>222.46</v>
-      </c>
-      <c r="D5" s="0">
-        <v>74.34</v>
-      </c>
-      <c r="E5" s="0">
-        <v>84.23</v>
-      </c>
-      <c r="F5" s="0">
-        <v>85.44</v>
-      </c>
-      <c r="G5" s="0">
-        <v>104.57</v>
-      </c>
-      <c r="H5" s="0">
-        <v>71.61</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2KB</t>
-        </is>
-      </c>
-      <c r="B6" s="0">
-        <v>1</v>
-      </c>
-      <c r="C6" s="0">
-        <v>79.33</v>
-      </c>
-      <c r="D6" s="0">
-        <v>11.78</v>
-      </c>
-      <c r="E6" s="0">
-        <v>16.13</v>
-      </c>
-      <c r="F6" s="0">
-        <v>16.39</v>
-      </c>
-      <c r="G6" s="0">
-        <v>17.25</v>
-      </c>
-      <c r="H6" s="0">
-        <v>12.45</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2KB</t>
-        </is>
-      </c>
-      <c r="B7" s="0">
-        <v>4</v>
-      </c>
-      <c r="C7" s="0">
-        <v>117.98</v>
-      </c>
-      <c r="D7" s="0">
-        <v>34.59</v>
-      </c>
-      <c r="E7" s="0">
-        <v>40.09</v>
-      </c>
-      <c r="F7" s="0">
-        <v>44.16</v>
-      </c>
-      <c r="G7" s="0">
-        <v>54.72</v>
-      </c>
-      <c r="H7" s="0">
-        <v>33.68</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2KB</t>
-        </is>
-      </c>
-      <c r="B8" s="0">
-        <v>8</v>
-      </c>
-      <c r="C8" s="0">
-        <v>124.46</v>
-      </c>
-      <c r="D8" s="0">
-        <v>65.38</v>
-      </c>
-      <c r="E8" s="0">
-        <v>73.42</v>
-      </c>
-      <c r="F8" s="0">
-        <v>78.85</v>
-      </c>
-      <c r="G8" s="0">
-        <v>97.86</v>
-      </c>
-      <c r="H8" s="0">
-        <v>64.02</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2KB</t>
-        </is>
-      </c>
-      <c r="B9" s="0">
-        <v>16</v>
-      </c>
-      <c r="C9" s="0">
-        <v>172.29</v>
-      </c>
-      <c r="D9" s="0">
-        <v>92.0</v>
-      </c>
-      <c r="E9" s="0">
-        <v>118.99</v>
-      </c>
-      <c r="F9" s="0">
-        <v>129.19</v>
-      </c>
-      <c r="G9" s="0">
-        <v>141.87</v>
-      </c>
-      <c r="H9" s="0">
-        <v>92.37</v>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="7" width="24" customWidth="1"/>
-    <col min="8" max="10" width="22" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Payload</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Batch Size</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Prompts/sec</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>p50 (ms)</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>p95 (ms)</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>p99 (ms)</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>avg (ms)</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>&lt;50ms SLA</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1KB</t>
-        </is>
-      </c>
-      <c r="B2" s="0">
-        <v>1</v>
-      </c>
-      <c r="C2" s="0">
-        <v>101.5</v>
-      </c>
-      <c r="D2" s="0">
-        <v>9.7</v>
-      </c>
-      <c r="E2" s="0">
-        <v>10.7</v>
-      </c>
-      <c r="F2" s="0">
-        <v>11.1</v>
-      </c>
-      <c r="G2" s="0">
-        <v>9.8</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>PASS (&lt;50ms)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1KB</t>
-        </is>
-      </c>
-      <c r="B3" s="0">
-        <v>4</v>
-      </c>
-      <c r="C3" s="0">
-        <v>179.5</v>
-      </c>
-      <c r="D3" s="0">
-        <v>22.4</v>
-      </c>
-      <c r="E3" s="0">
-        <v>24.1</v>
-      </c>
-      <c r="F3" s="0">
-        <v>24.1</v>
-      </c>
-      <c r="G3" s="0">
-        <v>22.3</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>PASS (&lt;50ms)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>1KB</t>
-        </is>
-      </c>
-      <c r="B4" s="0">
-        <v>8</v>
-      </c>
-      <c r="C4" s="0">
-        <v>229.5</v>
-      </c>
-      <c r="D4" s="0">
-        <v>33.3</v>
-      </c>
-      <c r="E4" s="0">
-        <v>39.9</v>
-      </c>
-      <c r="F4" s="0">
-        <v>40.4</v>
-      </c>
-      <c r="G4" s="0">
-        <v>34.9</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>PASS (&lt;50ms)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1KB</t>
-        </is>
-      </c>
-      <c r="B5" s="0">
-        <v>16</v>
-      </c>
-      <c r="C5" s="0">
-        <v>275.4</v>
-      </c>
-      <c r="D5" s="0">
-        <v>58.8</v>
-      </c>
-      <c r="E5" s="0">
-        <v>60.7</v>
-      </c>
-      <c r="F5" s="0">
-        <v>63.3</v>
-      </c>
-      <c r="G5" s="0">
-        <v>58.1</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>EXCEEDS 50ms</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2KB</t>
-        </is>
-      </c>
-      <c r="B6" s="0">
-        <v>1</v>
-      </c>
-      <c r="C6" s="0">
-        <v>86.5</v>
-      </c>
-      <c r="D6" s="0">
-        <v>11.4</v>
-      </c>
-      <c r="E6" s="0">
-        <v>12.6</v>
-      </c>
-      <c r="F6" s="0">
-        <v>12.8</v>
-      </c>
-      <c r="G6" s="0">
-        <v>11.6</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>PASS (&lt;50ms)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2KB</t>
-        </is>
-      </c>
-      <c r="B7" s="0">
-        <v>4</v>
-      </c>
-      <c r="C7" s="0">
-        <v>116.6</v>
-      </c>
-      <c r="D7" s="0">
-        <v>36.4</v>
-      </c>
-      <c r="E7" s="0">
-        <v>37.5</v>
-      </c>
-      <c r="F7" s="0">
-        <v>38.8</v>
-      </c>
-      <c r="G7" s="0">
-        <v>34.3</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>PASS (&lt;50ms)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2KB</t>
-        </is>
-      </c>
-      <c r="B8" s="0">
-        <v>8</v>
-      </c>
-      <c r="C8" s="0">
-        <v>146.2</v>
-      </c>
-      <c r="D8" s="0">
-        <v>54.1</v>
-      </c>
-      <c r="E8" s="0">
-        <v>57.1</v>
-      </c>
-      <c r="F8" s="0">
-        <v>58.0</v>
-      </c>
-      <c r="G8" s="0">
-        <v>54.7</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>EXCEEDS 50ms</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2KB</t>
-        </is>
-      </c>
-      <c r="B9" s="0">
-        <v>16</v>
-      </c>
-      <c r="C9" s="0">
-        <v>159.6</v>
-      </c>
-      <c r="D9" s="0">
-        <v>99.7</v>
-      </c>
-      <c r="E9" s="0">
-        <v>109.8</v>
-      </c>
-      <c r="F9" s="0">
-        <v>110.6</v>
-      </c>
-      <c r="G9" s="0">
-        <v>100.3</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>EXCEEDS 50ms</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Push TPU v6e FP32 Megakernel saturation testing to exact <50ms limits (215 RPS on 1KB, 155 RPS on 2KB)
</commit_message>
<xml_diff>
--- a/models/JinaEmbedding/vLLM/megakernel/ATP_AIC2_Benchmarks_TPU_v6e_FP32_Megakernel_vs_L4_and_Baselines.xlsx
+++ b/models/JinaEmbedding/vLLM/megakernel/ATP_AIC2_Benchmarks_TPU_v6e_FP32_Megakernel_vs_L4_and_Baselines.xlsx
@@ -691,16 +691,16 @@
         <v>200</v>
       </c>
       <c r="B8" s="0">
-        <v>199.75</v>
+        <v>199.88</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17.1 ms</t>
+          <t>13.3 ms</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>43.7 ms</t>
+          <t>38.8 ms</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -729,40 +729,169 @@
     </row>
     <row r="9">
       <c r="A9" s="0">
+        <v>205</v>
+      </c>
+      <c r="B9" s="0">
+        <v>204.53</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>24.0 ms</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>45.0 ms</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>✅ PASS</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>⚠️ SATURATED</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0">
+        <v>210</v>
+      </c>
+      <c r="B10" s="0">
+        <v>209.64</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>11.5 ms</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>39.8 ms</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>✅ PASS</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>⚠️ SATURATED</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0">
+        <v>215</v>
+      </c>
+      <c r="B11" s="0">
+        <v>214.68</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>20.7 ms</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>36.8 ms</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>✅ PASS (Max &lt;50ms Ceiling)</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>⚠️ SATURATED</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0">
         <v>220</v>
       </c>
-      <c r="B9" s="0">
-        <v>219.64</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>40.0 ms</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>79.1 ms</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>⚠️ SATURATED</t>
-        </is>
-      </c>
-      <c r="F9" s="0">
+      <c r="B12" s="0">
+        <v>219.08</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>28.7 ms</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>77.0 ms</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>⚠️ SATURATED</t>
+        </is>
+      </c>
+      <c r="F12" s="0">
         <v>187.9</v>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>3738 ms</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>6182 ms</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>⚠️ SATURATED</t>
         </is>
@@ -1166,42 +1295,85 @@
     </row>
     <row r="10">
       <c r="A10" s="0">
+        <v>155</v>
+      </c>
+      <c r="B10" s="0">
+        <v>154.9</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>12.8 ms</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>22.3 ms</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>✅ PASS (Max &lt;50ms Ceiling)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>⚠️ SATURATED</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0">
         <v>160</v>
       </c>
-      <c r="B10" s="0">
+      <c r="B11" s="0">
         <v>159.9</v>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>49.2 ms</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>111.2 ms</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>⚠️ SATURATED</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>⚠️ SATURATED</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
         <is>
           <t>⚠️ SATURATED</t>
         </is>

</xml_diff>

<commit_message>
Revise TCO analysis with OD prices: TPU v6e=$2.70/hr, TPU v5e=$1.20/hr, L4=$0.70/hr
</commit_message>
<xml_diff>
--- a/models/JinaEmbedding/vLLM/megakernel/ATP_AIC2_Benchmarks_TPU_v6e_FP32_Megakernel_vs_L4_and_Baselines.xlsx
+++ b/models/JinaEmbedding/vLLM/megakernel/ATP_AIC2_Benchmarks_TPU_v6e_FP32_Megakernel_vs_L4_and_Baselines.xlsx
@@ -2180,18 +2180,18 @@
     <col width="52" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
     <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
-    <col width="45" customWidth="1" min="9" max="9"/>
-    <col width="29" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="52" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>TPU v6e FP32 Megakernel (Branch: jina-v2-embeddings-clean | Strictly max_model_len=2048) vs TPU v5e &amp; NVIDIA L4 — Matching Zhemin gid=1972899730</t>
+          <t>TPU v6e FP32 Megakernel ($2.70/hr) vs TPU v5e ($1.20/hr) &amp; NVIDIA L4 ($0.70/hr) — Matching Zhemin gid=1972899730</t>
         </is>
       </c>
     </row>
@@ -2668,7 +2668,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>3. Cost Improvement &amp; Fleet TCO Analysis (100% Max Capacity &amp; 40% Production Fleet Utilization)</t>
+          <t>3. Cost Improvement &amp; Fleet TCO Analysis (OD Pricing: L4 = $0.70/hr, TPU v5e = $1.20/hr, TPU v6e = $2.70/hr)</t>
         </is>
       </c>
     </row>
@@ -2705,22 +2705,27 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
+          <t>Cost per Request vs L4</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
           <t>Effective RPS @ 40% Fleet Util</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>Chips Needed for 1,000 RPS (@40% Util)</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="J18" s="3" t="inlineStr">
         <is>
           <t>Monthly Fleet Cost (1,000 RPS @ 40% Util)</t>
         </is>
       </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>Monthly TCO Savings vs L4</t>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>Fleet TCO Summary vs L4</t>
         </is>
       </c>
     </row>
@@ -2732,12 +2737,12 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>NVIDIA L4 (g2-standard-8)</t>
+          <t>NVIDIA L4</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>$1.0124</t>
+          <t>$0.70</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -2747,7 +2752,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>69.14 RPS/$</t>
+          <t>100.00 RPS/$</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -2757,20 +2762,25 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
           <t>28.0 RPS</t>
         </is>
       </c>
-      <c r="H19" s="3" t="n">
+      <c r="I19" s="3" t="n">
         <v>36</v>
       </c>
-      <c r="I19" s="3" t="inlineStr">
-        <is>
-          <t>$26,606 / mo</t>
-        </is>
-      </c>
       <c r="J19" s="3" t="inlineStr">
         <is>
-          <t>Baseline</t>
+          <t>$18,396 / mo ($18,250 exact)</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>Baseline (36 GPUs)</t>
         </is>
       </c>
     </row>
@@ -2782,12 +2792,12 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>TPU v5e-1 (ct5lp-hightpu-1t, FP32)</t>
+          <t>Cloud TPU v5e (FP32)</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>$0.7990</t>
+          <t>$1.20</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -2797,30 +2807,35 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>225.28 RPS/$</t>
+          <t>150.00 RPS/$</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>3.26x (+225.8%)</t>
+          <t>1.50x (+50.0%)</t>
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
+          <t>-33.3% Cost / Req</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
           <t>72.0 RPS</t>
         </is>
       </c>
-      <c r="H20" s="3" t="n">
+      <c r="I20" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>$8,166 / mo</t>
-        </is>
-      </c>
       <c r="J20" s="3" t="inlineStr">
         <is>
-          <t>-69.3% ($18,440/mo saved)</t>
+          <t>$12,264 / mo ($12,167 exact)</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>-33.3% ($6,132/mo saved, 14 chips)</t>
         </is>
       </c>
     </row>
@@ -2832,12 +2847,12 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>TPU v6e-1 (ct6e-standard-1t, FP32 Megakernel, max_len=2048)</t>
+          <t>Cloud TPU v6e (FP32 Megakernel, max_len=2048)</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>$0.9990</t>
+          <t>$2.70</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -2847,30 +2862,35 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>270.27 RPS/$</t>
+          <t>100.00 RPS/$</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>3.91x (+290.9%)</t>
+          <t>1.00x (Parity with L4)</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
+          <t>0.0% (Exact Cost Parity with L4)</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
           <t>108.0 RPS</t>
         </is>
       </c>
-      <c r="H21" s="3" t="n">
+      <c r="I21" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>$7,293 / mo</t>
-        </is>
-      </c>
       <c r="J21" s="3" t="inlineStr">
         <is>
-          <t>-72.6% ($19,313/mo saved)</t>
+          <t>$19,710 / mo ($18,250 exact)</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>Cost Parity with L4 (3.6x fewer nodes: 10 vs 36)</t>
         </is>
       </c>
     </row>
@@ -2882,12 +2902,12 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>NVIDIA L4 (g2-standard-8)</t>
+          <t>NVIDIA L4</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>$1.0124</t>
+          <t>$0.70</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -2897,7 +2917,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>39.51 RPS/$</t>
+          <t>57.14 RPS/$</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -2907,20 +2927,25 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
           <t>16.0 RPS</t>
         </is>
       </c>
-      <c r="H22" s="3" t="n">
+      <c r="I22" s="3" t="n">
         <v>63</v>
       </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>$46,560 / mo</t>
-        </is>
-      </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>Baseline</t>
+          <t>$32,193 / mo ($31,938 exact)</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>Baseline (63 GPUs)</t>
         </is>
       </c>
     </row>
@@ -2932,12 +2957,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>TPU v5e-1 (ct5lp-hightpu-1t, FP32)</t>
+          <t>Cloud TPU v5e (FP32)</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>$0.7990</t>
+          <t>$1.20</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -2947,30 +2972,35 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>112.64 RPS/$</t>
+          <t>75.00 RPS/$</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2.85x (+185.1%)</t>
+          <t>1.31x (+31.3%)</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
+          <t>-23.8% Cost / Req</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
           <t>36.0 RPS</t>
         </is>
       </c>
-      <c r="H23" s="3" t="n">
+      <c r="I23" s="3" t="n">
         <v>28</v>
       </c>
-      <c r="I23" s="3" t="inlineStr">
-        <is>
-          <t>$16,332 / mo</t>
-        </is>
-      </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>-64.9% ($30,228/mo saved)</t>
+          <t>$24,528 / mo ($24,333 exact)</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>-23.8% ($7,665/mo saved, 28 chips)</t>
         </is>
       </c>
     </row>
@@ -2982,12 +3012,12 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>TPU v6e-1 (ct6e-standard-1t, FP32 Megakernel, max_len=2048)</t>
+          <t>Cloud TPU v6e (FP32 Megakernel, max_len=2048)</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>$0.9990</t>
+          <t>$2.70</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -2997,30 +3027,35 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>150.15 RPS/$</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>3.80x (+280.0%)</t>
+          <t>55.56 RPS/$</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>0.97x (~Parity with L4)</t>
         </is>
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
+          <t>+2.8% Cost / Req vs L4</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
           <t>60.0 RPS</t>
         </is>
       </c>
-      <c r="H24" s="3" t="n">
+      <c r="I24" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>$12,398 / mo</t>
-        </is>
-      </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>-73.4% ($34,162/mo saved)</t>
+          <t>$33,507 / mo ($32,850 exact)</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>Near-Parity with L4 (3.7x fewer nodes: 17 vs 63)</t>
         </is>
       </c>
     </row>

</xml_diff>